<commit_message>
Add portable NFC credential capabilities
</commit_message>
<xml_diff>
--- a/app/src/main/java/com/example/researchos/modules/nfc/docs/example_odk_nfc_tag_write.xlsx
+++ b/app/src/main/java/com/example/researchos/modules/nfc/docs/example_odk_nfc_tag_write.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R46a9e2559e1d4a3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="R7477f7a6f96b49c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Ra28f29b896cf427a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="Ra23823d2fcce49db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Rdd3cce0519364a7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R3fa9328afeca4e86"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -497,7 +497,7 @@
         <x:v>field-list</x:v>
       </x:c>
       <x:c r="I6" s="11" t="str">
-        <x:v>com.example.researchos.EXECUTE_METHOD(method_id='nfc_tag_write',input_value='${write_value}',input_record_type='text/plain',input_overwrite_policy=${overwrite_policy_input},input_expected_current_hash=${expected_current_hash_input},return_mode='flat')</x:v>
+        <x:v>com.example.researchos.EXECUTE_METHOD(method_id='nfc_tag_write',input_value=${write_value},input_record_type='text/plain',input_overwrite_policy=${overwrite_policy_input},input_expected_current_hash=${expected_current_hash_input},return_mode='flat')</x:v>
       </x:c>
       <x:c r="J6" s="11"/>
       <x:c r="K6" s="11"/>
@@ -952,7 +952,7 @@
         <x:v>nfc_tag_write</x:v>
       </x:c>
       <x:c r="C2" s="12" t="str">
-        <x:v>2026072707</x:v>
+        <x:v>2026072708</x:v>
       </x:c>
       <x:c r="D2" s="12" t="str">
         <x:v>${start}</x:v>

</xml_diff>